<commit_message>
Publish the current build
Synced by platform/publish_site.py, which checks the site against Files/outputs before and after.
</commit_message>
<xml_diff>
--- a/DATA_AUDIT.xlsx
+++ b/DATA_AUDIT.xlsx
@@ -8132,24 +8132,16 @@
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>PASS 2/4 - 2 FAIL</t>
-        </is>
-      </c>
-      <c r="G191" s="2" t="inlineStr">
-        <is>
-          <t>stage 5 missed programme rows the source contains</t>
-        </is>
-      </c>
-      <c r="H191" s="2" t="inlineStr">
-        <is>
-          <t>validation/recall_*.xlsx lists the candidates; widen the page range or split the document</t>
-        </is>
-      </c>
+          <t>PASS 4/4</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr"/>
+      <c r="H191" s="2" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -27084,32 +27076,24 @@
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E484" s="2" t="inlineStr">
         <is>
-          <t>900 row(s)</t>
+          <t>367 row(s)</t>
         </is>
       </c>
       <c r="F484" s="2" t="inlineStr">
         <is>
-          <t>65 duplicate key(s)</t>
-        </is>
-      </c>
-      <c r="G484" s="2" t="inlineStr">
-        <is>
-          <t>calcs, funding_by_program</t>
-        </is>
-      </c>
-      <c r="H484" s="2" t="inlineStr">
-        <is>
-          <t>a programme-year counted twice is a union key collision: check budget_row_id suffixes in budget_rows.csv</t>
-        </is>
-      </c>
+          <t>0 duplicate key(s)</t>
+        </is>
+      </c>
+      <c r="G484" s="2" t="inlineStr"/>
+      <c r="H484" s="2" t="inlineStr"/>
       <c r="I484" s="2" t="inlineStr">
         <is>
-          <t>["FY2022 head 1 programme 1.1 appears 2 times", "FY2022 head 2 programme 2.2 appears 2 times", "FY2022 head 3 programme 3.3 appears 2 times", "FY2022 head 4 programme 4.4 appears 2 times", "FY2022 head 5 programme 5.5 appears 2 times", "FY2022 head 6 programme 6.6 appears 2 times", "FY2024 head 1 programme 1.1 appears 2 times", "FY2024 head 2 programme 2.2 appears 2 times"]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -27136,7 +27120,7 @@
       </c>
       <c r="E485" s="2" t="inlineStr">
         <is>
-          <t>165 strategy-year(s)</t>
+          <t>35 strategy-year(s)</t>
         </is>
       </c>
       <c r="F485" s="2" t="inlineStr">
@@ -32336,27 +32320,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -32371,7 +32355,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>